<commit_message>
feat: Complete Milestone 3 - Remediation Agent, PR Summary Agent, RAG Assistant, Developer Review Portal, Report Exports (PDF/MD/JSON), and updated Excel project tracking documents
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -842,7 +842,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1081,6 +1081,174 @@
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Build Remediation Agent for specific fix recommendations &amp; corrected code snippets</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>US-08</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Build PR Summary Agent for executive review overview, health score &amp; prioritized roadmap</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Implement PDF, Markdown, and JSON Export Module for code review reports</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1106,7 +1274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W10"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1871,6 +2039,441 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>T-07</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Build Remediation Agent for fix recommendations &amp; corrected code examples</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AI Agent Dev</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>12</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>4</v>
+      </c>
+      <c r="U11" t="n">
+        <v>4</v>
+      </c>
+      <c r="V11" t="n">
+        <v>4</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>T-08</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Build PR Summary Agent for executive overview &amp; health score calculation</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AI Agent Dev</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>10</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>5</v>
+      </c>
+      <c r="V12" t="n">
+        <v>5</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>T-09</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Develop Developer Review Portal UI with severity filter &amp; interactive code viewer</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>14</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="n">
+        <v>7</v>
+      </c>
+      <c r="W13" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>US-15</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>T-10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>RAG &amp; Chat UI</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>12</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>T-11</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Implement PDF, Markdown, and JSON Code Review Report Generator &amp; Export Endpoints</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Reporting Dev</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:W1"/>
@@ -1886,7 +2489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2024,6 +2627,94 @@
       <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Started Next.js dev server (npm run dev) on port 3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Day 12</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Remediation agent corrected code formatting for Python &amp; Java</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Integrated standardized language templates for parameterized queries</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Day 13</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PR Summary Agent health score calculation precision across severities</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Implemented weighted health score formula max(0, 100 - weighted_sum)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Day 14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CORS preflight request blocked on frontend login endpoint</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Added allow_origin_regex in FastAPI main.py to allow all localhost origins</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Day 14</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Markdown and JSON export missing in report generator module</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Added generate_submission_markdown and generate_submission_json methods and routes</t>
         </is>
       </c>
     </row>
@@ -2215,22 +2906,22 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Full integration test runs</t>
+          <t>Full Milestone 3 multi-agent pipeline &amp; export endpoints</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Manual report formatting</t>
+          <t>Manual report formatting &amp; unhandled CORS options</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>End-to-end UI testing</t>
+          <t>Automated testing with pytest &amp; interactive developer portal</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Built automated PDF report generator</t>
+          <t>Completed Remediation Agent, PR Summary Agent, RAG Assistant &amp; PDF/MD/JSON exports</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
style: Cleanly align headers, cell borders, text wrapping, and column widths across all Excel project tracking documents
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,19 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -103,8 +114,20 @@
         <bgColor rgb="009BC2E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A8A"/>
+        <bgColor rgb="001E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -126,11 +149,25 @@
         <color rgb="00C0C0C0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,6 +197,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -530,725 +591,725 @@
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Planned Sprint</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Actual Sprint</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>US ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>User Story Description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>MOSCOW</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Dependency</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Assignee</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Study OWASP Top 10 guidelines &amp; security standards for Python/Java</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Design FastAPI backend architecture, SQLAlchemy models and API router</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Implement Code Submission Module (Paste &amp; Upload endpoints)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Implement AST &amp; Regex Language Auto-Detection for Python and Java</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="12" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Build ChromaDB RAG Vector Knowledge Base with HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Build Code Analysis Agent for quality, complexity &amp; anti-patterns</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>US-07</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Build Security Vulnerability Agent for OWASP Top 10 (CWE-798, CWE-89)</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Build LangGraph multi-agent parallel execution orchestrator pipeline</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>US-06, US-07</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>US-09</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Validate multi-agent pipeline using vulnerable sample code suites</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Build Next.js Dashboard UI &amp; Security Findings Display Panel</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr">
         <is>
           <t>US-11</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Implement RAG Assistant search interface &amp; API vector store query endpoint</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>US-12</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>Implement PDF &amp; HTML Executive Summary Report Generator</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Could</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="13" t="inlineStr">
         <is>
           <t>Build Remediation Agent for specific fix recommendations &amp; corrected code snippets</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Build PR Summary Agent for executive review overview, health score &amp; prioritized roadmap</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>Implement PDF, Markdown, and JSON Export Module for code review reports</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="14" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1277,1200 +1338,1244 @@
   <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-    <col width="7" customWidth="1" min="18" max="18"/>
-    <col width="7" customWidth="1" min="19" max="19"/>
-    <col width="7" customWidth="1" min="20" max="20"/>
-    <col width="7" customWidth="1" min="21" max="21"/>
-    <col width="7" customWidth="1" min="22" max="22"/>
-    <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>NOTES: Task sizing should be between 0.5 to 12 hours</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="11" t="n"/>
+      <c r="K1" s="11" t="n"/>
+      <c r="L1" s="11" t="n"/>
+      <c r="M1" s="11" t="n"/>
+      <c r="N1" s="11" t="n"/>
+      <c r="O1" s="11" t="n"/>
+      <c r="P1" s="11" t="n"/>
+      <c r="Q1" s="11" t="n"/>
+      <c r="R1" s="11" t="n"/>
+      <c r="S1" s="11" t="n"/>
+      <c r="T1" s="11" t="n"/>
+      <c r="U1" s="11" t="n"/>
+      <c r="V1" s="11" t="n"/>
+      <c r="W1" s="11" t="n"/>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>US ID</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Task ID</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>Task Description</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Task Start Date</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Task Completion Date</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Team Member</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>Original Estimate Effort (In Hours)</t>
         </is>
       </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>Day1</t>
         </is>
       </c>
-      <c r="K2" s="7" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>Day2</t>
         </is>
       </c>
-      <c r="L2" s="7" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>Day3</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="M2" s="12" t="inlineStr">
         <is>
           <t>Day4</t>
         </is>
       </c>
-      <c r="N2" s="7" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>Day5</t>
         </is>
       </c>
-      <c r="O2" s="7" t="inlineStr">
+      <c r="O2" s="12" t="inlineStr">
         <is>
           <t>Day6</t>
         </is>
       </c>
-      <c r="P2" s="7" t="inlineStr">
+      <c r="P2" s="12" t="inlineStr">
         <is>
           <t>Day7</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
+      <c r="Q2" s="12" t="inlineStr">
         <is>
           <t>Day8</t>
         </is>
       </c>
-      <c r="R2" s="7" t="inlineStr">
+      <c r="R2" s="12" t="inlineStr">
         <is>
           <t>Day9</t>
         </is>
       </c>
-      <c r="S2" s="7" t="inlineStr">
+      <c r="S2" s="12" t="inlineStr">
         <is>
           <t>Day10</t>
         </is>
       </c>
-      <c r="T2" s="7" t="inlineStr">
+      <c r="T2" s="12" t="inlineStr">
         <is>
           <t>Day11</t>
         </is>
       </c>
-      <c r="U2" s="7" t="inlineStr">
+      <c r="U2" s="12" t="inlineStr">
         <is>
           <t>Day12</t>
         </is>
       </c>
-      <c r="V2" s="7" t="inlineStr">
+      <c r="V2" s="12" t="inlineStr">
         <is>
           <t>Day13</t>
         </is>
       </c>
-      <c r="W2" s="7" t="inlineStr">
+      <c r="W2" s="12" t="inlineStr">
         <is>
           <t>Day14</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="6" t="inlineStr"/>
-      <c r="B3" s="6" t="inlineStr"/>
-      <c r="C3" s="6" t="inlineStr"/>
-      <c r="D3" s="6" t="inlineStr"/>
-      <c r="E3" s="6" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="6" t="inlineStr"/>
-      <c r="H3" s="6" t="inlineStr"/>
-      <c r="I3" s="7">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="16" t="inlineStr"/>
+      <c r="B3" s="16" t="inlineStr"/>
+      <c r="C3" s="17" t="inlineStr"/>
+      <c r="D3" s="16" t="inlineStr"/>
+      <c r="E3" s="16" t="inlineStr"/>
+      <c r="F3" s="17" t="inlineStr"/>
+      <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr"/>
+      <c r="I3" s="18">
         <f>SUM(I5:I20)</f>
         <v/>
       </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
+      <c r="L3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M3" s="7" t="inlineStr">
+      <c r="M3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N3" s="7" t="inlineStr">
+      <c r="N3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" s="7" t="inlineStr">
+      <c r="O3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" s="7" t="inlineStr">
+      <c r="P3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="Q3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
+      <c r="R3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="S3" s="7" t="inlineStr">
+      <c r="S3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T3" s="7" t="inlineStr">
+      <c r="T3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U3" s="7" t="inlineStr">
+      <c r="U3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="V3" s="7" t="inlineStr">
+      <c r="V3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="W3" s="7" t="inlineStr">
+      <c r="W3" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="12" t="n"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n"/>
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="12" t="n"/>
+      <c r="L4" s="12" t="n"/>
+      <c r="M4" s="12" t="n"/>
+      <c r="N4" s="12" t="n"/>
+      <c r="O4" s="12" t="n"/>
+      <c r="P4" s="12" t="n"/>
+      <c r="Q4" s="12" t="n"/>
+      <c r="R4" s="12" t="n"/>
+      <c r="S4" s="12" t="n"/>
+      <c r="T4" s="12" t="n"/>
+      <c r="U4" s="12" t="n"/>
+      <c r="V4" s="12" t="n"/>
+      <c r="W4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>Research OWASP Top 10 guidelines &amp; security standards</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="3" t="n">
+      <c r="J5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="K5" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="L5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Design FastAPI backend architecture and DB schemas</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="3" t="n">
+      <c r="J6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="3" t="n">
+      <c r="L6" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="M6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="M6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>T-03</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Implement Code Submission Paste &amp; Upload APIs</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="J7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="3" t="n">
+      <c r="J7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="N7" s="3" t="n">
+      <c r="N7" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="O7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="O7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Implement Python &amp; Java AST language detector</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="3" t="n">
+      <c r="J8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="P8" s="3" t="n">
+      <c r="P8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="Q8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="Q8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Setup ChromaDB vector store and HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr">
         <is>
           <t>RAG Setup</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="J9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="3" t="n">
+      <c r="J9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="R9" s="3" t="n">
+      <c r="R9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="S9" s="3" t="n">
+      <c r="S9" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="T9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="T9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Implement Code Analysis Agent for quality &amp; smells</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="J10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="3" t="n">
+      <c r="J10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="U10" s="3" t="n">
+      <c r="U10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="3" t="n">
+      <c r="V10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="W10" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="W10" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>T-07</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>Build Remediation Agent for fix recommendations &amp; corrected code examples</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="14" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="14" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
+      <c r="J11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="U11" t="n">
+      <c r="U11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="V11" t="n">
+      <c r="V11" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="W11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="W11" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>T-08</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Build PR Summary Agent for executive overview &amp; health score calculation</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="n">
+      <c r="J12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="V12" t="n">
+      <c r="V12" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="W12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="W12" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>T-09</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Develop Developer Review Portal UI with severity filter &amp; interactive code viewer</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Frontend Dev</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="n">
+      <c r="J13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="W13" t="n">
+      <c r="W13" s="14" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="13" t="inlineStr">
         <is>
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>RAG &amp; Chat UI</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" t="n">
+      <c r="J14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="12" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>T-11</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Implement PDF, Markdown, and JSON Code Review Report Generator &amp; Export Endpoints</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Reporting Dev</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="I15" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" t="n">
+      <c r="J15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="14" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2492,227 +2597,227 @@
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C1" s="9" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Impediments</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Action Taken</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>FastAPI router duplicate endpoint registration</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="13" t="inlineStr">
         <is>
           <t>Cleaned router.py and removed duplicate route bindings</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>Anthropic API key dependency issue</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="15" t="inlineStr">
         <is>
           <t>Migrated orchestrator model calls to Google Gemini API</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Day 5</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Missing virtual environment packages during setup</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Updated requirements.txt and reinstalled backend venv</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Day 8</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>ChromaDB vector store timeout on RAG search</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Fixed backend server connection and initialized embeddings</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Day 10</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Next.js frontend connection refused on port 3000</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Started Next.js dev server (npm run dev) on port 3000</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>Day 12</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Remediation agent corrected code formatting for Python &amp; Java</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Integrated standardized language templates for parameterized queries</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Day 13</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>PR Summary Agent health score calculation precision across severities</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Implemented weighted health score formula max(0, 100 - weighted_sum)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Day 14</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>CORS preflight request blocked on frontend login endpoint</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Added allow_origin_regex in FastAPI main.py to allow all localhost origins</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Day 14</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Markdown and JSON export missing in report generator module</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added generate_submission_markdown and generate_submission_json methods and routes</t>
         </is>
@@ -2734,192 +2839,192 @@
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>SL #</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Sprint #</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>Sprint start date</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Sprint end date</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Team member name</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Start Doing</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Stop Doing</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Continue Doing</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Action taken</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="3" t="n">
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Automated AST syntax checking</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="13" t="inlineStr">
         <is>
           <t>Hardcoding API endpoints</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="13" t="inlineStr">
         <is>
           <t>Writing modular agent code</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="13" t="inlineStr">
         <is>
           <t>Established centralized config.py</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="34" customHeight="1">
-      <c r="A3" s="3" t="n">
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="14" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="15" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Parallel LangGraph execution</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Synchronous vector DB calls</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>Comprehensive unit testing</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>Implemented async ChromaDB retriever</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="3" t="n">
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Full Milestone 3 multi-agent pipeline &amp; export endpoints</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Manual report formatting &amp; unhandled CORS options</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>Automated testing with pytest &amp; interactive developer portal</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="13" t="inlineStr">
         <is>
           <t>Completed Remediation Agent, PR Summary Agent, RAG Assistant &amp; PDF/MD/JSON exports</t>
         </is>

</xml_diff>

<commit_message>
refactor: Update Sprint 3 dates in Excel project tracking documents to reflect 2-week July timeline (2026-07-16 to 2026-07-29)
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -127,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -163,11 +163,55 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -223,6 +267,8 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1369,28 +1415,28 @@
           <t>NOTES: Task sizing should be between 0.5 to 12 hours</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="11" t="n"/>
-      <c r="H1" s="11" t="n"/>
-      <c r="I1" s="11" t="n"/>
-      <c r="J1" s="11" t="n"/>
-      <c r="K1" s="11" t="n"/>
-      <c r="L1" s="11" t="n"/>
-      <c r="M1" s="11" t="n"/>
-      <c r="N1" s="11" t="n"/>
-      <c r="O1" s="11" t="n"/>
-      <c r="P1" s="11" t="n"/>
-      <c r="Q1" s="11" t="n"/>
-      <c r="R1" s="11" t="n"/>
-      <c r="S1" s="11" t="n"/>
-      <c r="T1" s="11" t="n"/>
-      <c r="U1" s="11" t="n"/>
-      <c r="V1" s="11" t="n"/>
-      <c r="W1" s="11" t="n"/>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
+      <c r="D1" s="19" t="n"/>
+      <c r="E1" s="19" t="n"/>
+      <c r="F1" s="19" t="n"/>
+      <c r="G1" s="19" t="n"/>
+      <c r="H1" s="19" t="n"/>
+      <c r="I1" s="19" t="n"/>
+      <c r="J1" s="19" t="n"/>
+      <c r="K1" s="19" t="n"/>
+      <c r="L1" s="19" t="n"/>
+      <c r="M1" s="19" t="n"/>
+      <c r="N1" s="19" t="n"/>
+      <c r="O1" s="19" t="n"/>
+      <c r="P1" s="19" t="n"/>
+      <c r="Q1" s="19" t="n"/>
+      <c r="R1" s="19" t="n"/>
+      <c r="S1" s="19" t="n"/>
+      <c r="T1" s="19" t="n"/>
+      <c r="U1" s="19" t="n"/>
+      <c r="V1" s="19" t="n"/>
+      <c r="W1" s="20" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
@@ -1599,28 +1645,28 @@
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="13" t="n"/>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-      <c r="Q4" s="12" t="n"/>
-      <c r="R4" s="12" t="n"/>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
-      <c r="U4" s="12" t="n"/>
-      <c r="V4" s="12" t="n"/>
-      <c r="W4" s="12" t="n"/>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
+      <c r="L4" s="19" t="n"/>
+      <c r="M4" s="19" t="n"/>
+      <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
+      <c r="P4" s="19" t="n"/>
+      <c r="Q4" s="19" t="n"/>
+      <c r="R4" s="19" t="n"/>
+      <c r="S4" s="19" t="n"/>
+      <c r="T4" s="19" t="n"/>
+      <c r="U4" s="19" t="n"/>
+      <c r="V4" s="19" t="n"/>
+      <c r="W4" s="20" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -2162,12 +2208,12 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
@@ -2249,12 +2295,12 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
@@ -2336,12 +2382,12 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
@@ -2423,12 +2469,12 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -2510,12 +2556,12 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -3001,7 +3047,7 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">

</xml_diff>

<commit_message>
refactor: Update Sprint 3 dates in Excel project tracking documents to reflect past two weeks leading to today (2026-07-25 to 2026-08-07)
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -2208,12 +2208,12 @@
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="F13" s="15" t="inlineStr">
@@ -2469,12 +2469,12 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
@@ -2556,12 +2556,12 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
@@ -3042,12 +3042,12 @@
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">

</xml_diff>

<commit_message>
feat: Add additional user stories US-17-20, tasks T-12-15, standups, defects 11-13, and test cases 19-20 to Excel tracking workbooks
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1356,6 +1356,174 @@
         </is>
       </c>
       <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Implement JWT Authentication &amp; User Dashboard Session Management</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>US-02</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>US-18</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Integrate Interactive Line-by-Line Code Viewer with Color-Coded Vulnerability Highlights</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Implement 1-Click Complete Refactored Source Code Copy &amp; Download Engine</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="G20" s="13" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>US-20</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Build Automated Pytest Suite &amp; E2E System Integration Verification Script</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1381,7 +1549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1390,7 +1558,7 @@
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="35" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -1415,28 +1583,28 @@
           <t>NOTES: Task sizing should be between 0.5 to 12 hours</t>
         </is>
       </c>
-      <c r="B1" s="19" t="n"/>
-      <c r="C1" s="19" t="n"/>
-      <c r="D1" s="19" t="n"/>
-      <c r="E1" s="19" t="n"/>
-      <c r="F1" s="19" t="n"/>
-      <c r="G1" s="19" t="n"/>
-      <c r="H1" s="19" t="n"/>
-      <c r="I1" s="19" t="n"/>
-      <c r="J1" s="19" t="n"/>
-      <c r="K1" s="19" t="n"/>
-      <c r="L1" s="19" t="n"/>
-      <c r="M1" s="19" t="n"/>
-      <c r="N1" s="19" t="n"/>
-      <c r="O1" s="19" t="n"/>
-      <c r="P1" s="19" t="n"/>
-      <c r="Q1" s="19" t="n"/>
-      <c r="R1" s="19" t="n"/>
-      <c r="S1" s="19" t="n"/>
-      <c r="T1" s="19" t="n"/>
-      <c r="U1" s="19" t="n"/>
-      <c r="V1" s="19" t="n"/>
-      <c r="W1" s="20" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="11" t="n"/>
+      <c r="E1" s="11" t="n"/>
+      <c r="F1" s="11" t="n"/>
+      <c r="G1" s="11" t="n"/>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="11" t="n"/>
+      <c r="K1" s="11" t="n"/>
+      <c r="L1" s="11" t="n"/>
+      <c r="M1" s="11" t="n"/>
+      <c r="N1" s="11" t="n"/>
+      <c r="O1" s="11" t="n"/>
+      <c r="P1" s="11" t="n"/>
+      <c r="Q1" s="11" t="n"/>
+      <c r="R1" s="11" t="n"/>
+      <c r="S1" s="11" t="n"/>
+      <c r="T1" s="11" t="n"/>
+      <c r="U1" s="11" t="n"/>
+      <c r="V1" s="11" t="n"/>
+      <c r="W1" s="11" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="12" t="inlineStr">
@@ -1645,28 +1813,28 @@
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n"/>
-      <c r="C4" s="19" t="n"/>
-      <c r="D4" s="19" t="n"/>
-      <c r="E4" s="19" t="n"/>
-      <c r="F4" s="19" t="n"/>
-      <c r="G4" s="19" t="n"/>
-      <c r="H4" s="19" t="n"/>
-      <c r="I4" s="19" t="n"/>
-      <c r="J4" s="19" t="n"/>
-      <c r="K4" s="19" t="n"/>
-      <c r="L4" s="19" t="n"/>
-      <c r="M4" s="19" t="n"/>
-      <c r="N4" s="19" t="n"/>
-      <c r="O4" s="19" t="n"/>
-      <c r="P4" s="19" t="n"/>
-      <c r="Q4" s="19" t="n"/>
-      <c r="R4" s="19" t="n"/>
-      <c r="S4" s="19" t="n"/>
-      <c r="T4" s="19" t="n"/>
-      <c r="U4" s="19" t="n"/>
-      <c r="V4" s="19" t="n"/>
-      <c r="W4" s="20" t="n"/>
+      <c r="B4" s="12" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="12" t="n"/>
+      <c r="E4" s="12" t="n"/>
+      <c r="F4" s="13" t="n"/>
+      <c r="G4" s="12" t="n"/>
+      <c r="H4" s="12" t="n"/>
+      <c r="I4" s="12" t="n"/>
+      <c r="J4" s="12" t="n"/>
+      <c r="K4" s="12" t="n"/>
+      <c r="L4" s="12" t="n"/>
+      <c r="M4" s="12" t="n"/>
+      <c r="N4" s="12" t="n"/>
+      <c r="O4" s="12" t="n"/>
+      <c r="P4" s="12" t="n"/>
+      <c r="Q4" s="12" t="n"/>
+      <c r="R4" s="12" t="n"/>
+      <c r="S4" s="12" t="n"/>
+      <c r="T4" s="12" t="n"/>
+      <c r="U4" s="12" t="n"/>
+      <c r="V4" s="12" t="n"/>
+      <c r="W4" s="12" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -2623,6 +2791,354 @@
       </c>
       <c r="W15" s="14" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>T-12</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Implement Password Hashing (bcrypt) &amp; JWT Access Token Router Endpoints</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Auth &amp; Security</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="U16" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="V16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>US-18</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>T-13</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>Build Line-by-Line Code Viewer with Severity Filter Chips (Critical, High, Medium, Low)</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>Frontend UI</t>
+        </is>
+      </c>
+      <c r="H17" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="V17" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="W17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>T-14</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Implement Complete Refactored Source File Generator &amp; Full Remediated Code Tab</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Agent &amp; UI Dev</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="W18" s="12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>US-20</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>T-15</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Develop Automated Pytest Unit &amp; End-to-End Integration Suite (18 Test Cases)</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>QA &amp; Testing</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="14" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2640,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2866,6 +3382,72 @@
       <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added generate_submission_markdown and generate_submission_json methods and routes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>JWT Token expiration handling on user dashboard refresh</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Configured auth context state persistence in localStorage</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>Day 6</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>High cyclomatic complexity display on long functions</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Implemented AST node depth counter and cognitive complexity metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Day 9</t>
+        </is>
+      </c>
+      <c r="C13" s="15" t="inlineStr">
+        <is>
+          <t>ChromaDB vector store connection timeout during RAG query</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr">
+        <is>
+          <t>Added connection pool retry logic and fallback grounded search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update project title, MIT license copyright, formatted excel sheets, and Milestone 4 enhancements
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -269,6 +269,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -634,16 +646,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -690,840 +702,1008 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Study OWASP Top 10 guidelines &amp; security standards for Python/Java</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Design FastAPI backend architecture, SQLAlchemy models and API router</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F3" s="15" t="inlineStr">
+      <c r="F3" s="21" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="G3" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H3" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Implement Code Submission Module (Paste &amp; Upload endpoints)</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Implement AST &amp; Regex Language Auto-Detection for Python and Java</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Build ChromaDB RAG Vector Knowledge Base with HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="21" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>Build Code Analysis Agent for quality, complexity &amp; anti-patterns</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
+      <c r="F7" s="21" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="G7" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>US-07</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>Build Security Vulnerability Agent for OWASP Top 10 (CWE-798, CWE-89)</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Build LangGraph multi-agent parallel execution orchestrator pipeline</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr">
         <is>
           <t>US-06, US-07</t>
         </is>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>US-09</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>Validate multi-agent pipeline using vulnerable sample code suites</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="21" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Build Next.js Dashboard UI &amp; Security Findings Display Panel</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="F11" s="21" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="G11" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>US-11</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Implement RAG Assistant search interface &amp; API vector store query endpoint</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="21" t="inlineStr">
         <is>
           <t>US-12</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Implement PDF &amp; HTML Executive Summary Report Generator</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>Could</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="F13" s="21" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Build Remediation Agent for specific fix recommendations &amp; corrected code snippets</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Build PR Summary Agent for executive review overview, health score &amp; prioritized roadmap</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F15" s="15" t="inlineStr">
+      <c r="F15" s="21" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="21" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>Implement PDF, Markdown, and JSON Export Module for code review reports</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F17" s="21" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="G17" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="21" t="inlineStr">
         <is>
           <t>US-17</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Implement JWT Authentication &amp; User Dashboard Session Management</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="21" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="21" t="inlineStr">
         <is>
           <t>US-18</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>Integrate Interactive Line-by-Line Code Viewer with Color-Coded Vulnerability Highlights</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F19" s="21" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
       </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="G19" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="21" t="inlineStr">
         <is>
           <t>US-19</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Implement 1-Click Complete Refactored Source Code Copy &amp; Download Engine</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
+      <c r="F20" s="21" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="G20" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H20" s="12" t="inlineStr">
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="21" t="inlineStr">
         <is>
           <t>US-20</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>Build Automated Pytest Suite &amp; E2E System Integration Verification Script</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="21" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F21" s="15" t="inlineStr">
+      <c r="F21" s="21" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>US-21</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>Implement Post-Generation Remediation Validator for AST and syntax validation of generated code</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>US-13</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Implement Side-by-Side Code Diff Viewer for interactive before-and-after PR comparisons</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F23" s="21" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>US-23</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>Implement Dynamic Security Policy Filter for real-time finding persistence and threshold controls</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>US-10</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C25" s="21" t="inlineStr">
+        <is>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>Update Project Title to 'Development of Smart Code Inspection Platform with Vulnerability Detection System Group 2' and add MIT License</t>
+        </is>
+      </c>
+      <c r="E25" s="21" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="F25" s="21" t="inlineStr">
+        <is>
+          <t>US-16</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1549,32 +1729,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1583,1561 +1763,1909 @@
           <t>NOTES: Task sizing should be between 0.5 to 12 hours</t>
         </is>
       </c>
-      <c r="B1" s="11" t="n"/>
-      <c r="C1" s="11" t="n"/>
-      <c r="D1" s="11" t="n"/>
-      <c r="E1" s="11" t="n"/>
-      <c r="F1" s="11" t="n"/>
-      <c r="G1" s="11" t="n"/>
-      <c r="H1" s="11" t="n"/>
-      <c r="I1" s="11" t="n"/>
-      <c r="J1" s="11" t="n"/>
-      <c r="K1" s="11" t="n"/>
-      <c r="L1" s="11" t="n"/>
-      <c r="M1" s="11" t="n"/>
-      <c r="N1" s="11" t="n"/>
-      <c r="O1" s="11" t="n"/>
-      <c r="P1" s="11" t="n"/>
-      <c r="Q1" s="11" t="n"/>
-      <c r="R1" s="11" t="n"/>
-      <c r="S1" s="11" t="n"/>
-      <c r="T1" s="11" t="n"/>
-      <c r="U1" s="11" t="n"/>
-      <c r="V1" s="11" t="n"/>
-      <c r="W1" s="11" t="n"/>
+      <c r="B1" s="23" t="n"/>
+      <c r="C1" s="23" t="n"/>
+      <c r="D1" s="23" t="n"/>
+      <c r="E1" s="23" t="n"/>
+      <c r="F1" s="23" t="n"/>
+      <c r="G1" s="23" t="n"/>
+      <c r="H1" s="23" t="n"/>
+      <c r="I1" s="23" t="n"/>
+      <c r="J1" s="23" t="n"/>
+      <c r="K1" s="23" t="n"/>
+      <c r="L1" s="23" t="n"/>
+      <c r="M1" s="23" t="n"/>
+      <c r="N1" s="23" t="n"/>
+      <c r="O1" s="23" t="n"/>
+      <c r="P1" s="23" t="n"/>
+      <c r="Q1" s="23" t="n"/>
+      <c r="R1" s="23" t="n"/>
+      <c r="S1" s="23" t="n"/>
+      <c r="T1" s="23" t="n"/>
+      <c r="U1" s="23" t="n"/>
+      <c r="V1" s="23" t="n"/>
+      <c r="W1" s="24" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>US ID</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Task ID</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Task Description</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Task Start Date</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>Task Completion Date</t>
         </is>
       </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>Team Member</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Activity</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>Original Estimate Effort (In Hours)</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="22" t="inlineStr">
         <is>
           <t>Day1</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="22" t="inlineStr">
         <is>
           <t>Day2</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="22" t="inlineStr">
         <is>
           <t>Day3</t>
         </is>
       </c>
-      <c r="M2" s="12" t="inlineStr">
+      <c r="M2" s="22" t="inlineStr">
         <is>
           <t>Day4</t>
         </is>
       </c>
-      <c r="N2" s="12" t="inlineStr">
+      <c r="N2" s="22" t="inlineStr">
         <is>
           <t>Day5</t>
         </is>
       </c>
-      <c r="O2" s="12" t="inlineStr">
+      <c r="O2" s="22" t="inlineStr">
         <is>
           <t>Day6</t>
         </is>
       </c>
-      <c r="P2" s="12" t="inlineStr">
+      <c r="P2" s="22" t="inlineStr">
         <is>
           <t>Day7</t>
         </is>
       </c>
-      <c r="Q2" s="12" t="inlineStr">
+      <c r="Q2" s="22" t="inlineStr">
         <is>
           <t>Day8</t>
         </is>
       </c>
-      <c r="R2" s="12" t="inlineStr">
+      <c r="R2" s="22" t="inlineStr">
         <is>
           <t>Day9</t>
         </is>
       </c>
-      <c r="S2" s="12" t="inlineStr">
+      <c r="S2" s="22" t="inlineStr">
         <is>
           <t>Day10</t>
         </is>
       </c>
-      <c r="T2" s="12" t="inlineStr">
+      <c r="T2" s="22" t="inlineStr">
         <is>
           <t>Day11</t>
         </is>
       </c>
-      <c r="U2" s="12" t="inlineStr">
+      <c r="U2" s="22" t="inlineStr">
         <is>
           <t>Day12</t>
         </is>
       </c>
-      <c r="V2" s="12" t="inlineStr">
+      <c r="V2" s="22" t="inlineStr">
         <is>
           <t>Day13</t>
         </is>
       </c>
-      <c r="W2" s="12" t="inlineStr">
+      <c r="W2" s="22" t="inlineStr">
         <is>
           <t>Day14</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="16" t="inlineStr"/>
-      <c r="B3" s="16" t="inlineStr"/>
-      <c r="C3" s="17" t="inlineStr"/>
-      <c r="D3" s="16" t="inlineStr"/>
-      <c r="E3" s="16" t="inlineStr"/>
-      <c r="F3" s="17" t="inlineStr"/>
-      <c r="G3" s="16" t="inlineStr"/>
-      <c r="H3" s="16" t="inlineStr"/>
-      <c r="I3" s="18">
+      <c r="A3" s="22" t="inlineStr"/>
+      <c r="B3" s="22" t="inlineStr"/>
+      <c r="C3" s="22" t="inlineStr"/>
+      <c r="D3" s="22" t="inlineStr"/>
+      <c r="E3" s="22" t="inlineStr"/>
+      <c r="F3" s="22" t="inlineStr"/>
+      <c r="G3" s="22" t="inlineStr"/>
+      <c r="H3" s="22" t="inlineStr"/>
+      <c r="I3" s="22">
         <f>SUM(I5:I20)</f>
         <v/>
       </c>
-      <c r="J3" s="18" t="inlineStr">
+      <c r="J3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K3" s="18" t="inlineStr">
+      <c r="K3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L3" s="18" t="inlineStr">
+      <c r="L3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M3" s="18" t="inlineStr">
+      <c r="M3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N3" s="18" t="inlineStr">
+      <c r="N3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" s="18" t="inlineStr">
+      <c r="O3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" s="18" t="inlineStr">
+      <c r="P3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q3" s="18" t="inlineStr">
+      <c r="Q3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R3" s="18" t="inlineStr">
+      <c r="R3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="S3" s="18" t="inlineStr">
+      <c r="S3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T3" s="18" t="inlineStr">
+      <c r="T3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U3" s="18" t="inlineStr">
+      <c r="U3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="V3" s="18" t="inlineStr">
+      <c r="V3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="W3" s="18" t="inlineStr">
+      <c r="W3" s="21" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n"/>
-      <c r="C4" s="13" t="n"/>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="12" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-      <c r="J4" s="12" t="n"/>
-      <c r="K4" s="12" t="n"/>
-      <c r="L4" s="12" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="12" t="n"/>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-      <c r="Q4" s="12" t="n"/>
-      <c r="R4" s="12" t="n"/>
-      <c r="S4" s="12" t="n"/>
-      <c r="T4" s="12" t="n"/>
-      <c r="U4" s="12" t="n"/>
-      <c r="V4" s="12" t="n"/>
-      <c r="W4" s="12" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+      <c r="G4" s="22" t="n"/>
+      <c r="H4" s="22" t="n"/>
+      <c r="I4" s="22" t="n"/>
+      <c r="J4" s="22" t="n"/>
+      <c r="K4" s="22" t="n"/>
+      <c r="L4" s="22" t="n"/>
+      <c r="M4" s="22" t="n"/>
+      <c r="N4" s="22" t="n"/>
+      <c r="O4" s="22" t="n"/>
+      <c r="P4" s="22" t="n"/>
+      <c r="Q4" s="22" t="n"/>
+      <c r="R4" s="22" t="n"/>
+      <c r="S4" s="22" t="n"/>
+      <c r="T4" s="22" t="n"/>
+      <c r="U4" s="22" t="n"/>
+      <c r="V4" s="22" t="n"/>
+      <c r="W4" s="22" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Research OWASP Top 10 guidelines &amp; security standards</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Research</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I5" s="14" t="n">
+      <c r="I5" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="K5" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="14" t="n">
+      <c r="L5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Design FastAPI backend architecture and DB schemas</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="21" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>Architecture</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="12" t="n">
+      <c r="J6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="M6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="12" t="n">
+      <c r="M6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>T-03</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Implement Code Submission Paste &amp; Upload APIs</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="F7" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="H7" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I7" s="14" t="n">
+      <c r="I7" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="14" t="n">
+      <c r="J7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="N7" s="14" t="n">
+      <c r="N7" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="O7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="14" t="n">
+      <c r="O7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Implement Python &amp; Java AST language detector</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="21" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
         <is>
           <t>Development</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="H8" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="12" t="n">
+      <c r="J8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="P8" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="Q8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="12" t="n">
+      <c r="Q8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Setup ChromaDB vector store and HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="F9" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
         <is>
           <t>RAG Setup</t>
         </is>
       </c>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="H9" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I9" s="14" t="n">
+      <c r="I9" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="14" t="n">
+      <c r="J9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="R9" s="14" t="n">
+      <c r="R9" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="S9" s="14" t="n">
+      <c r="S9" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="T9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" s="14" t="n">
+      <c r="T9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Implement Code Analysis Agent for quality &amp; smells</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="21" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="H10" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="12" t="n">
+      <c r="J10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="U10" s="12" t="n">
+      <c r="U10" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="12" t="n">
+      <c r="V10" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="W10" s="12" t="n">
+      <c r="W10" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>T-07</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>Build Remediation Agent for fix recommendations &amp; corrected code examples</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="21" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I11" s="14" t="n">
+      <c r="I11" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="14" t="n">
+      <c r="J11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="U11" s="14" t="n">
+      <c r="U11" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="V11" s="14" t="n">
+      <c r="V11" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="W11" s="14" t="n">
+      <c r="W11" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>T-08</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Build PR Summary Agent for executive overview &amp; health score calculation</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="21" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="12" t="n">
+      <c r="J12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="V12" s="12" t="n">
+      <c r="V12" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="W12" s="12" t="n">
+      <c r="W12" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>T-09</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Develop Developer Review Portal UI with severity filter &amp; interactive code viewer</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="21" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="21" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Frontend Dev</t>
         </is>
       </c>
-      <c r="H13" s="14" t="inlineStr">
+      <c r="H13" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I13" s="14" t="n">
+      <c r="I13" s="21" t="n">
         <v>14</v>
       </c>
-      <c r="J13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="14" t="n">
+      <c r="J13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="W13" s="14" t="n">
+      <c r="W13" s="21" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="21" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>RAG &amp; Chat UI</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="I14" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="12" t="n">
+      <c r="J14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="21" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>T-11</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Implement PDF, Markdown, and JSON Code Review Report Generator &amp; Export Endpoints</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="21" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="21" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="F15" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>Reporting Dev</t>
         </is>
       </c>
-      <c r="H15" s="14" t="inlineStr">
+      <c r="H15" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I15" s="14" t="n">
+      <c r="I15" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" s="14" t="n">
+      <c r="J15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>US-17</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>T-12</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Implement Password Hashing (bcrypt) &amp; JWT Access Token Router Endpoints</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="21" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Auth &amp; Security</t>
         </is>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I16" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="12" t="n">
+      <c r="J16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="U16" s="12" t="n">
+      <c r="U16" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="V16" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="12" t="n">
+      <c r="V16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>US-18</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>T-13</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Build Line-by-Line Code Viewer with Severity Filter Chips (Critical, High, Medium, Low)</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="21" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="21" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G17" s="22" t="inlineStr">
         <is>
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H17" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I17" s="14" t="n">
+      <c r="I17" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="J17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" s="14" t="n">
+      <c r="J17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="V17" s="14" t="n">
+      <c r="V17" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="W17" s="14" t="n">
+      <c r="W17" s="21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>US-19</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>T-14</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>Implement Complete Refactored Source File Generator &amp; Full Remediated Code Tab</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="21" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
         <is>
           <t>Agent &amp; UI Dev</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr">
+      <c r="H18" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="J18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" s="12" t="n">
+      <c r="J18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="W18" s="12" t="n">
+      <c r="W18" s="21" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>US-20</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>T-15</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>Develop Automated Pytest Unit &amp; End-to-End Integration Suite (18 Test Cases)</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="21" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G19" s="22" t="inlineStr">
         <is>
           <t>QA &amp; Testing</t>
         </is>
       </c>
-      <c r="H19" s="14" t="inlineStr">
+      <c r="H19" s="21" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I19" s="14" t="n">
+      <c r="I19" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="J19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="14" t="n">
+      <c r="J19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="21" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>US-21</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>T-16</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>Build Post-Generation Remediation Validator for AST check</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>Validation Dev</t>
+        </is>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I20" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="J20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="U20" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="V20" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>T-17</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>Integrate Side-by-Side Code Diff Viewer in PR Summary view</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F21" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G21" s="22" t="inlineStr">
+        <is>
+          <t>Frontend UI</t>
+        </is>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="J21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="V21" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="W21" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>US-23</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>T-18</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>Build Dynamic Security Policy Filtering Engine for interactive portal views</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Security Policy</t>
+        </is>
+      </c>
+      <c r="H22" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I22" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="J22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="W22" s="21" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>US-24</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>T-19</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>Update Project Branding &amp; Title and integrate MIT License across docs and app</t>
+        </is>
+      </c>
+      <c r="D23" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="E23" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Branding &amp; Legal</t>
+        </is>
+      </c>
+      <c r="H23" s="21" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="I23" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="21" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3156,13 +3684,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3188,266 +3716,354 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>FastAPI router duplicate endpoint registration</t>
         </is>
       </c>
-      <c r="D2" s="13" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Cleaned router.py and removed duplicate route bindings</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>Anthropic API key dependency issue</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>Migrated orchestrator model calls to Google Gemini API</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Day 5</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Missing virtual environment packages during setup</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>Updated requirements.txt and reinstalled backend venv</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Day 8</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>ChromaDB vector store timeout on RAG search</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Fixed backend server connection and initialized embeddings</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Day 10</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Next.js frontend connection refused on port 3000</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Started Next.js dev server (npm run dev) on port 3000</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Day 12</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Remediation agent corrected code formatting for Python &amp; Java</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>Integrated standardized language templates for parameterized queries</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Day 13</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>PR Summary Agent health score calculation precision across severities</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>Implemented weighted health score formula max(0, 100 - weighted_sum)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Day 14</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>CORS preflight request blocked on frontend login endpoint</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Added allow_origin_regex in FastAPI main.py to allow all localhost origins</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Day 14</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Markdown and JSON export missing in report generator module</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>Added generate_submission_markdown and generate_submission_json methods and routes</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>JWT Token expiration handling on user dashboard refresh</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Configured auth context state persistence in localStorage</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Day 6</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>High cyclomatic complexity display on long functions</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Implemented AST node depth counter and cognitive complexity metrics</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Day 9</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>ChromaDB vector store connection timeout during RAG query</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Added connection pool retry logic and fallback grounded search</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>LLM remediation generated syntax warnings on edge case imports</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>Created AST Post-Generation Remediation Validator to guarantee syntactically sound fixes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>PR review summary needed visual diff comparison between original and fixed code</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Integrated side-by-side code diff viewer component into PR Summary tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Day 5</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
+        <is>
+          <t>Security policy toggle was not dynamically updating finding counters</t>
+        </is>
+      </c>
+      <c r="D16" s="22" t="inlineStr">
+        <is>
+          <t>Connected Security Policy state store to portal findings filter</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Day 7</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
+        <is>
+          <t>Project title update required across backend API, frontend UI, report generators, and license</t>
+        </is>
+      </c>
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>Updated title to 'Development of Smart Code Inspection Platform with Vulnerability Detection System Group 2' and created MIT LICENSE file</t>
         </is>
       </c>
     </row>
@@ -3462,17 +4078,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -3524,137 +4140,182 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="12" t="n">
+      <c r="A2" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="21" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="21" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="21" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>Automated AST syntax checking</t>
         </is>
       </c>
-      <c r="G2" s="13" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>Hardcoding API endpoints</t>
         </is>
       </c>
-      <c r="H2" s="13" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>Writing modular agent code</t>
         </is>
       </c>
-      <c r="I2" s="13" t="inlineStr">
+      <c r="I2" s="22" t="inlineStr">
         <is>
           <t>Established centralized config.py</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="14" t="n">
+      <c r="A3" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="21" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="21" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D3" s="14" t="inlineStr">
+      <c r="D3" s="21" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="F3" s="15" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>Parallel LangGraph execution</t>
         </is>
       </c>
-      <c r="G3" s="15" t="inlineStr">
+      <c r="G3" s="22" t="inlineStr">
         <is>
           <t>Synchronous vector DB calls</t>
         </is>
       </c>
-      <c r="H3" s="15" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Comprehensive unit testing</t>
         </is>
       </c>
-      <c r="I3" s="15" t="inlineStr">
+      <c r="I3" s="22" t="inlineStr">
         <is>
           <t>Implemented async ChromaDB retriever</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>Thimmampalli Asritha</t>
-        </is>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>Full Milestone 3 multi-agent pipeline &amp; export endpoints</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G4" s="22" t="inlineStr">
         <is>
           <t>Manual report formatting &amp; unhandled CORS options</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Automated testing with pytest &amp; interactive developer portal</t>
         </is>
       </c>
-      <c r="I4" s="13" t="inlineStr">
+      <c r="I4" s="22" t="inlineStr">
         <is>
           <t>Completed Remediation Agent, PR Summary Agent, RAG Assistant &amp; PDF/MD/JSON exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Thimmampalli Asritha</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>Strict AST validation for LLM output &amp; dynamic security policies</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>Unvalidated code snippet generation &amp; hardcoded project branding</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>End-to-end integration testing &amp; standard documentation compliance</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>Completed Milestone 4 pipeline hardening, code diff viewer, dynamic security policies, MIT License, and title branding</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Enhance security portal, chatbot handling, and format excel documentation
</commit_message>
<xml_diff>
--- a/Agile_Template_v0.1.xlsx
+++ b/Agile_Template_v0.1.xlsx
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -280,6 +280,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -649,70 +652,70 @@
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Planned Sprint</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Actual Sprint</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>US ID</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>User Story Description</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>MOSCOW</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="25" t="inlineStr">
         <is>
           <t>Dependency</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>Assignee</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="H1" s="25" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
@@ -722,7 +725,7 @@
           <t>Study OWASP Top 10 guidelines &amp; security standards for Python/Java</t>
         </is>
       </c>
-      <c r="E2" s="21" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
@@ -737,24 +740,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H2" s="21" t="inlineStr">
+      <c r="H2" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
@@ -764,12 +767,12 @@
           <t>Design FastAPI backend architecture, SQLAlchemy models and API router</t>
         </is>
       </c>
-      <c r="E3" s="21" t="inlineStr">
+      <c r="E3" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F3" s="21" t="inlineStr">
+      <c r="F3" s="22" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
@@ -779,24 +782,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H3" s="21" t="inlineStr">
+      <c r="H3" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
@@ -806,12 +809,12 @@
           <t>Implement Code Submission Module (Paste &amp; Upload endpoints)</t>
         </is>
       </c>
-      <c r="E4" s="21" t="inlineStr">
+      <c r="E4" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F4" s="21" t="inlineStr">
+      <c r="F4" s="22" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
@@ -821,24 +824,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
@@ -848,12 +851,12 @@
           <t>Implement AST &amp; Regex Language Auto-Detection for Python and Java</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
@@ -863,24 +866,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C6" s="21" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
@@ -890,12 +893,12 @@
           <t>Build ChromaDB RAG Vector Knowledge Base with HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F6" s="21" t="inlineStr">
+      <c r="F6" s="22" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
@@ -905,24 +908,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C7" s="21" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
@@ -932,12 +935,12 @@
           <t>Build Code Analysis Agent for quality, complexity &amp; anti-patterns</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
@@ -947,24 +950,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>US-07</t>
         </is>
@@ -974,12 +977,12 @@
           <t>Build Security Vulnerability Agent for OWASP Top 10 (CWE-798, CWE-89)</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
@@ -989,24 +992,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
@@ -1016,12 +1019,12 @@
           <t>Build LangGraph multi-agent parallel execution orchestrator pipeline</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>US-06, US-07</t>
         </is>
@@ -1031,24 +1034,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>US-09</t>
         </is>
@@ -1058,12 +1061,12 @@
           <t>Validate multi-agent pipeline using vulnerable sample code suites</t>
         </is>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F10" s="21" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
@@ -1073,24 +1076,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H10" s="21" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C11" s="21" t="inlineStr">
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1100,12 +1103,12 @@
           <t>Build Next.js Dashboard UI &amp; Security Findings Display Panel</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
@@ -1115,24 +1118,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>US-11</t>
         </is>
@@ -1142,12 +1145,12 @@
           <t>Implement RAG Assistant search interface &amp; API vector store query endpoint</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Should</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1157,24 +1160,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C13" s="21" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>US-12</t>
         </is>
@@ -1184,12 +1187,12 @@
           <t>Implement PDF &amp; HTML Executive Summary Report Generator</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>Could</t>
         </is>
       </c>
-      <c r="F13" s="21" t="inlineStr">
+      <c r="F13" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1199,24 +1202,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C14" s="21" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
@@ -1226,12 +1229,12 @@
           <t>Build Remediation Agent for specific fix recommendations &amp; corrected code snippets</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>US-08</t>
         </is>
@@ -1241,24 +1244,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C15" s="21" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
@@ -1268,12 +1271,12 @@
           <t>Build PR Summary Agent for executive review overview, health score &amp; prioritized roadmap</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
@@ -1283,24 +1286,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H15" s="21" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C16" s="21" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
@@ -1310,12 +1313,12 @@
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1325,24 +1328,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
@@ -1352,12 +1355,12 @@
           <t>Implement PDF, Markdown, and JSON Export Module for code review reports</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F17" s="21" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
@@ -1367,24 +1370,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>US-17</t>
         </is>
@@ -1394,12 +1397,12 @@
           <t>Implement JWT Authentication &amp; User Dashboard Session Management</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F18" s="21" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
@@ -1409,24 +1412,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C19" s="21" t="inlineStr">
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>US-18</t>
         </is>
@@ -1436,12 +1439,12 @@
           <t>Integrate Interactive Line-by-Line Code Viewer with Color-Coded Vulnerability Highlights</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="F19" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1451,24 +1454,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C20" s="21" t="inlineStr">
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>US-19</t>
         </is>
@@ -1478,12 +1481,12 @@
           <t>Implement 1-Click Complete Refactored Source Code Copy &amp; Download Engine</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F20" s="21" t="inlineStr">
+      <c r="F20" s="22" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
@@ -1493,24 +1496,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>US-20</t>
         </is>
@@ -1520,12 +1523,12 @@
           <t>Build Automated Pytest Suite &amp; E2E System Integration Verification Script</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
@@ -1535,24 +1538,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C22" s="21" t="inlineStr">
+      <c r="C22" s="22" t="inlineStr">
         <is>
           <t>US-21</t>
         </is>
@@ -1562,12 +1565,12 @@
           <t>Implement Post-Generation Remediation Validator for AST and syntax validation of generated code</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
@@ -1577,24 +1580,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C23" s="21" t="inlineStr">
+      <c r="C23" s="22" t="inlineStr">
         <is>
           <t>US-22</t>
         </is>
@@ -1604,12 +1607,12 @@
           <t>Implement Side-by-Side Code Diff Viewer for interactive before-and-after PR comparisons</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F23" s="21" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1619,24 +1622,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H23" s="21" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B24" s="21" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C24" s="21" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>US-23</t>
         </is>
@@ -1646,12 +1649,12 @@
           <t>Implement Dynamic Security Policy Filter for real-time finding persistence and threshold controls</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F24" s="22" t="inlineStr">
         <is>
           <t>US-10</t>
         </is>
@@ -1661,24 +1664,24 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
+      <c r="H24" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
+      <c r="A25" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B25" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C25" s="21" t="inlineStr">
+      <c r="C25" s="22" t="inlineStr">
         <is>
           <t>US-24</t>
         </is>
@@ -1688,12 +1691,12 @@
           <t>Update Project Title to 'Development of Smart Code Inspection Platform with Vulnerability Detection System Group 2' and add MIT License</t>
         </is>
       </c>
-      <c r="E25" s="21" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>Must</t>
         </is>
       </c>
-      <c r="F25" s="21" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
@@ -1703,7 +1706,7 @@
           <t>Thimmampalli Asritha</t>
         </is>
       </c>
-      <c r="H25" s="21" t="inlineStr">
+      <c r="H25" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -1732,59 +1735,59 @@
   <dimension ref="A1:W23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="38" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
-    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="37" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>NOTES: Task sizing should be between 0.5 to 12 hours</t>
         </is>
       </c>
-      <c r="B1" s="23" t="n"/>
-      <c r="C1" s="23" t="n"/>
-      <c r="D1" s="23" t="n"/>
-      <c r="E1" s="23" t="n"/>
-      <c r="F1" s="23" t="n"/>
-      <c r="G1" s="23" t="n"/>
-      <c r="H1" s="23" t="n"/>
-      <c r="I1" s="23" t="n"/>
-      <c r="J1" s="23" t="n"/>
-      <c r="K1" s="23" t="n"/>
-      <c r="L1" s="23" t="n"/>
-      <c r="M1" s="23" t="n"/>
-      <c r="N1" s="23" t="n"/>
-      <c r="O1" s="23" t="n"/>
-      <c r="P1" s="23" t="n"/>
-      <c r="Q1" s="23" t="n"/>
-      <c r="R1" s="23" t="n"/>
-      <c r="S1" s="23" t="n"/>
-      <c r="T1" s="23" t="n"/>
-      <c r="U1" s="23" t="n"/>
-      <c r="V1" s="23" t="n"/>
-      <c r="W1" s="24" t="n"/>
+      <c r="B1" s="19" t="n"/>
+      <c r="C1" s="19" t="n"/>
+      <c r="D1" s="19" t="n"/>
+      <c r="E1" s="19" t="n"/>
+      <c r="F1" s="19" t="n"/>
+      <c r="G1" s="19" t="n"/>
+      <c r="H1" s="19" t="n"/>
+      <c r="I1" s="19" t="n"/>
+      <c r="J1" s="19" t="n"/>
+      <c r="K1" s="19" t="n"/>
+      <c r="L1" s="19" t="n"/>
+      <c r="M1" s="19" t="n"/>
+      <c r="N1" s="19" t="n"/>
+      <c r="O1" s="19" t="n"/>
+      <c r="P1" s="19" t="n"/>
+      <c r="Q1" s="19" t="n"/>
+      <c r="R1" s="19" t="n"/>
+      <c r="S1" s="19" t="n"/>
+      <c r="T1" s="19" t="n"/>
+      <c r="U1" s="19" t="n"/>
+      <c r="V1" s="19" t="n"/>
+      <c r="W1" s="20" t="n"/>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="22" t="inlineStr">
@@ -1916,72 +1919,72 @@
         <f>SUM(I5:I20)</f>
         <v/>
       </c>
-      <c r="J3" s="21" t="inlineStr">
+      <c r="J3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="K3" s="21" t="inlineStr">
+      <c r="K3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="L3" s="21" t="inlineStr">
+      <c r="L3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M3" s="21" t="inlineStr">
+      <c r="M3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="N3" s="21" t="inlineStr">
+      <c r="N3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" s="21" t="inlineStr">
+      <c r="O3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" s="21" t="inlineStr">
+      <c r="P3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Q3" s="21" t="inlineStr">
+      <c r="Q3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="R3" s="21" t="inlineStr">
+      <c r="R3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="S3" s="21" t="inlineStr">
+      <c r="S3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="T3" s="21" t="inlineStr">
+      <c r="T3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U3" s="21" t="inlineStr">
+      <c r="U3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="V3" s="21" t="inlineStr">
+      <c r="V3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="W3" s="21" t="inlineStr">
+      <c r="W3" s="22" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1993,36 +1996,36 @@
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-      <c r="B4" s="22" t="n"/>
-      <c r="C4" s="22" t="n"/>
-      <c r="D4" s="22" t="n"/>
-      <c r="E4" s="22" t="n"/>
-      <c r="F4" s="22" t="n"/>
-      <c r="G4" s="22" t="n"/>
-      <c r="H4" s="22" t="n"/>
-      <c r="I4" s="22" t="n"/>
-      <c r="J4" s="22" t="n"/>
-      <c r="K4" s="22" t="n"/>
-      <c r="L4" s="22" t="n"/>
-      <c r="M4" s="22" t="n"/>
-      <c r="N4" s="22" t="n"/>
-      <c r="O4" s="22" t="n"/>
-      <c r="P4" s="22" t="n"/>
-      <c r="Q4" s="22" t="n"/>
-      <c r="R4" s="22" t="n"/>
-      <c r="S4" s="22" t="n"/>
-      <c r="T4" s="22" t="n"/>
-      <c r="U4" s="22" t="n"/>
-      <c r="V4" s="22" t="n"/>
-      <c r="W4" s="22" t="n"/>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
+      <c r="I4" s="19" t="n"/>
+      <c r="J4" s="19" t="n"/>
+      <c r="K4" s="19" t="n"/>
+      <c r="L4" s="19" t="n"/>
+      <c r="M4" s="19" t="n"/>
+      <c r="N4" s="19" t="n"/>
+      <c r="O4" s="19" t="n"/>
+      <c r="P4" s="19" t="n"/>
+      <c r="Q4" s="19" t="n"/>
+      <c r="R4" s="19" t="n"/>
+      <c r="S4" s="19" t="n"/>
+      <c r="T4" s="19" t="n"/>
+      <c r="U4" s="19" t="n"/>
+      <c r="V4" s="19" t="n"/>
+      <c r="W4" s="20" t="n"/>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>US-01</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>T-01</t>
         </is>
@@ -2032,12 +2035,12 @@
           <t>Research OWASP Top 10 guidelines &amp; security standards</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
@@ -2052,64 +2055,64 @@
           <t>Research</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="21" t="n">
+      <c r="K5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="L5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="21" t="n">
+      <c r="L5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>US-02</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>T-02</t>
         </is>
@@ -2119,12 +2122,12 @@
           <t>Design FastAPI backend architecture and DB schemas</t>
         </is>
       </c>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
@@ -2139,64 +2142,64 @@
           <t>Architecture</t>
         </is>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="21" t="n">
+      <c r="J6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="L6" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="M6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" s="21" t="n">
+      <c r="M6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>US-03</t>
         </is>
       </c>
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>T-03</t>
         </is>
@@ -2206,12 +2209,12 @@
           <t>Implement Code Submission Paste &amp; Upload APIs</t>
         </is>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="E7" s="21" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
@@ -2226,64 +2229,64 @@
           <t>Development</t>
         </is>
       </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" s="21" t="n">
+      <c r="J7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="O7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" s="21" t="n">
+      <c r="O7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>US-04</t>
         </is>
       </c>
-      <c r="B8" s="21" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>T-04</t>
         </is>
@@ -2293,12 +2296,12 @@
           <t>Implement Python &amp; Java AST language detector</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
@@ -2313,64 +2316,64 @@
           <t>Development</t>
         </is>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="J8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="21" t="n">
+      <c r="J8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="P8" s="21" t="n">
+      <c r="P8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="Q8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" s="21" t="n">
+      <c r="Q8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>US-05</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>T-05</t>
         </is>
@@ -2380,12 +2383,12 @@
           <t>Setup ChromaDB vector store and HuggingFace embeddings</t>
         </is>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="E9" s="21" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
@@ -2400,64 +2403,64 @@
           <t>RAG Setup</t>
         </is>
       </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="21" t="n">
+      <c r="J9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="R9" s="21" t="n">
+      <c r="R9" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="S9" s="21" t="n">
+      <c r="S9" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="T9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" s="21" t="n">
+      <c r="T9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>US-06</t>
         </is>
       </c>
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>T-06</t>
         </is>
@@ -2467,12 +2470,12 @@
           <t>Implement Code Analysis Agent for quality &amp; smells</t>
         </is>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>2026-07-11</t>
         </is>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
@@ -2487,64 +2490,64 @@
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H10" s="21" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="21" t="n">
+      <c r="J10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="U10" s="21" t="n">
+      <c r="U10" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="21" t="n">
+      <c r="V10" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="W10" s="21" t="n">
+      <c r="W10" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>US-13</t>
         </is>
       </c>
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>T-07</t>
         </is>
@@ -2554,12 +2557,12 @@
           <t>Build Remediation Agent for fix recommendations &amp; corrected code examples</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="E11" s="21" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
@@ -2574,64 +2577,64 @@
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H11" s="21" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="21" t="n">
+      <c r="J11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="U11" s="21" t="n">
+      <c r="U11" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="V11" s="21" t="n">
+      <c r="V11" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="W11" s="21" t="n">
+      <c r="W11" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>US-14</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>T-08</t>
         </is>
@@ -2641,12 +2644,12 @@
           <t>Build PR Summary Agent for executive overview &amp; health score calculation</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
@@ -2661,64 +2664,64 @@
           <t>AI Agent Dev</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="21" t="n">
+      <c r="J12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="V12" s="21" t="n">
+      <c r="V12" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="W12" s="21" t="n">
+      <c r="W12" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>T-09</t>
         </is>
@@ -2728,12 +2731,12 @@
           <t>Develop Developer Review Portal UI with severity filter &amp; interactive code viewer</t>
         </is>
       </c>
-      <c r="D13" s="21" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
@@ -2748,64 +2751,64 @@
           <t>Frontend Dev</t>
         </is>
       </c>
-      <c r="H13" s="21" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="J13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="21" t="n">
+      <c r="J13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="W13" s="21" t="n">
+      <c r="W13" s="22" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>US-15</t>
         </is>
       </c>
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>T-10</t>
         </is>
@@ -2815,12 +2818,12 @@
           <t>Build RAG Conversational Code Assistant interface &amp; ChromaDB query integration</t>
         </is>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
@@ -2835,64 +2838,64 @@
           <t>RAG &amp; Chat UI</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="21" t="n">
+      <c r="J14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>US-16</t>
         </is>
       </c>
-      <c r="B15" s="21" t="inlineStr">
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>T-11</t>
         </is>
@@ -2902,12 +2905,12 @@
           <t>Implement PDF, Markdown, and JSON Code Review Report Generator &amp; Export Endpoints</t>
         </is>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="E15" s="22" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -2922,64 +2925,64 @@
           <t>Reporting Dev</t>
         </is>
       </c>
-      <c r="H15" s="21" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I15" s="21" t="n">
+      <c r="I15" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" s="21" t="n">
+      <c r="J15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V15" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>US-17</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>T-12</t>
         </is>
@@ -2989,12 +2992,12 @@
           <t>Implement Password Hashing (bcrypt) &amp; JWT Access Token Router Endpoints</t>
         </is>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>2026-07-26</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
@@ -3009,64 +3012,64 @@
           <t>Auth &amp; Security</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I16" s="21" t="n">
+      <c r="I16" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="21" t="n">
+      <c r="J16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="U16" s="21" t="n">
+      <c r="U16" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="V16" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="21" t="n">
+      <c r="V16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>US-18</t>
         </is>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>T-13</t>
         </is>
@@ -3076,12 +3079,12 @@
           <t>Build Line-by-Line Code Viewer with Severity Filter Chips (Critical, High, Medium, Low)</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="E17" s="21" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
@@ -3096,64 +3099,64 @@
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="H17" s="21" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I17" s="21" t="n">
+      <c r="I17" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U17" s="21" t="n">
+      <c r="J17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="V17" s="21" t="n">
+      <c r="V17" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="W17" s="21" t="n">
+      <c r="W17" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>US-19</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>T-14</t>
         </is>
@@ -3163,12 +3166,12 @@
           <t>Implement Complete Refactored Source File Generator &amp; Full Remediated Code Tab</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
@@ -3183,64 +3186,64 @@
           <t>Agent &amp; UI Dev</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I18" s="21" t="n">
+      <c r="I18" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" s="21" t="n">
+      <c r="J18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U18" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V18" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="W18" s="21" t="n">
+      <c r="W18" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>US-20</t>
         </is>
       </c>
-      <c r="B19" s="21" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>T-15</t>
         </is>
@@ -3250,12 +3253,12 @@
           <t>Develop Automated Pytest Unit &amp; End-to-End Integration Suite (18 Test Cases)</t>
         </is>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -3270,64 +3273,64 @@
           <t>QA &amp; Testing</t>
         </is>
       </c>
-      <c r="H19" s="21" t="inlineStr">
+      <c r="H19" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I19" s="21" t="n">
+      <c r="I19" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="J19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W19" s="21" t="n">
+      <c r="J19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>US-21</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>T-16</t>
         </is>
@@ -3337,12 +3340,12 @@
           <t>Build Post-Generation Remediation Validator for AST check</t>
         </is>
       </c>
-      <c r="D20" s="21" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
@@ -3357,64 +3360,64 @@
           <t>Validation Dev</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I20" s="21" t="n">
+      <c r="I20" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="21" t="n">
+      <c r="J20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="U20" s="21" t="n">
+      <c r="U20" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="V20" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" s="21" t="n">
+      <c r="V20" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>US-22</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>T-17</t>
         </is>
@@ -3424,12 +3427,12 @@
           <t>Integrate Side-by-Side Code Diff Viewer in PR Summary view</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>2026-08-13</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
@@ -3444,64 +3447,64 @@
           <t>Frontend UI</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I21" s="21" t="n">
+      <c r="I21" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="J21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U21" s="21" t="n">
+      <c r="J21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="V21" s="21" t="n">
+      <c r="V21" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="W21" s="21" t="n">
+      <c r="W21" s="22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>US-23</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>T-18</t>
         </is>
@@ -3511,12 +3514,12 @@
           <t>Build Dynamic Security Policy Filtering Engine for interactive portal views</t>
         </is>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>2026-08-15</t>
         </is>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>2026-08-16</t>
         </is>
@@ -3531,64 +3534,64 @@
           <t>Security Policy</t>
         </is>
       </c>
-      <c r="H22" s="21" t="inlineStr">
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I22" s="21" t="n">
+      <c r="I22" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="J22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" s="21" t="n">
+      <c r="J22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V22" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="W22" s="21" t="n">
+      <c r="W22" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>US-24</t>
         </is>
       </c>
-      <c r="B23" s="21" t="inlineStr">
+      <c r="B23" s="22" t="inlineStr">
         <is>
           <t>T-19</t>
         </is>
@@ -3598,12 +3601,12 @@
           <t>Update Project Branding &amp; Title and integrate MIT License across docs and app</t>
         </is>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>
@@ -3618,54 +3621,54 @@
           <t>Branding &amp; Legal</t>
         </is>
       </c>
-      <c r="H23" s="21" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I23" s="21" t="n">
+      <c r="I23" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="J23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="U23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" s="21" t="n">
-        <v>0</v>
-      </c>
-      <c r="W23" s="21" t="n">
+      <c r="J23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="V23" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W23" s="22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3687,36 +3690,36 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>Impediments</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>Action Taken</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
@@ -3738,7 +3741,7 @@
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
@@ -3760,7 +3763,7 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
@@ -3782,7 +3785,7 @@
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
@@ -3804,7 +3807,7 @@
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3826,7 +3829,7 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3848,7 +3851,7 @@
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="21" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3870,7 +3873,7 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3892,7 +3895,7 @@
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3914,7 +3917,7 @@
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3936,7 +3939,7 @@
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3958,7 +3961,7 @@
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
@@ -3980,7 +3983,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -4002,7 +4005,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -4024,7 +4027,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -4046,7 +4049,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
@@ -4081,79 +4084,79 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>SL #</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="25" t="inlineStr">
         <is>
           <t>Sprint #</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="25" t="inlineStr">
         <is>
           <t>Sprint start date</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="25" t="inlineStr">
         <is>
           <t>Sprint end date</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="25" t="inlineStr">
         <is>
           <t>Team member name</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="25" t="inlineStr">
         <is>
           <t>Start Doing</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="G1" s="25" t="inlineStr">
         <is>
           <t>Stop Doing</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="H1" s="25" t="inlineStr">
         <is>
           <t>Continue Doing</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="I1" s="25" t="inlineStr">
         <is>
           <t>Action taken</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="21" t="n">
+      <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="21" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C2" s="21" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="D2" s="21" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
@@ -4185,20 +4188,20 @@
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="21" t="n">
+      <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="21" t="inlineStr">
+      <c r="B3" s="22" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="C3" s="21" t="inlineStr">
+      <c r="C3" s="22" t="inlineStr">
         <is>
           <t>2026-07-08</t>
         </is>
       </c>
-      <c r="D3" s="21" t="inlineStr">
+      <c r="D3" s="22" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
@@ -4230,20 +4233,20 @@
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="21" t="n">
+      <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="D4" s="22" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
@@ -4275,20 +4278,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>2026-08-08</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>2026-08-17</t>
         </is>

</xml_diff>